<commit_message>
fix: hashtag_fetch reads its temp JSON as UTF-8 (accented names were double-encoded)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/src/data/hashtag_2026-10-29.xlsx
+++ b/src/data/hashtag_2026-10-29.xlsx
@@ -3501,7 +3501,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Alperen SengÃ¼n</t>
+          <t>Alperen Sengün</t>
         </is>
       </c>
       <c r="C48" t="n">
@@ -11466,7 +11466,7 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>Dennis SchrÃ¶der</t>
+          <t>Dennis Schröder</t>
         </is>
       </c>
       <c r="C171" t="inlineStr"/>
@@ -11592,7 +11592,7 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>Moussa DiabatÃ©</t>
+          <t>Moussa Diabaté</t>
         </is>
       </c>
       <c r="C173" t="n">
@@ -19340,7 +19340,7 @@
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>Hugo GonzÃ¡lez</t>
+          <t>Hugo González</t>
         </is>
       </c>
       <c r="C295" t="inlineStr"/>
@@ -20033,7 +20033,7 @@
       </c>
       <c r="B306" t="inlineStr">
         <is>
-          <t>VÃ­t KrejcÃ­</t>
+          <t>Vít Krejcí</t>
         </is>
       </c>
       <c r="C306" t="inlineStr"/>
@@ -20474,7 +20474,7 @@
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t>Nolan TraorÃ©</t>
+          <t>Nolan Traoré</t>
         </is>
       </c>
       <c r="C313" t="inlineStr"/>
@@ -26008,7 +26008,7 @@
       </c>
       <c r="B401" t="inlineStr">
         <is>
-          <t>Tidjane SalaÃ¼n</t>
+          <t>Tidjane Salaün</t>
         </is>
       </c>
       <c r="C401" t="inlineStr"/>
@@ -27396,7 +27396,7 @@
       </c>
       <c r="B423" t="inlineStr">
         <is>
-          <t>PacÃ´me Dadiet</t>
+          <t>Pacôme Dadiet</t>
         </is>
       </c>
       <c r="C423" t="inlineStr"/>

</xml_diff>